<commit_message>
add funtions color, propensity
</commit_message>
<xml_diff>
--- a/data/radar_template.xlsx
+++ b/data/radar_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,11 @@
           <t>linkName</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>propensityToWin</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -466,7 +471,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -508,7 +513,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Less Than 1 Year</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -550,7 +555,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1-3 Years</t>
+          <t>Beyond This Year</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -573,10 +578,40 @@
           <t>quantum, research, innovation</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Applications</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;br&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Propensity" error="Please select from the list" type="list">
+      <formula1>"Low,Medium,High"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>